<commit_message>
atualização de layout e tela de onboarding
</commit_message>
<xml_diff>
--- a/concursoai_roadmap_v3_FINAL.xlsx
+++ b/concursoai_roadmap_v3_FINAL.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="54">
+  <fonts count="55">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -329,6 +329,11 @@
       <color rgb="00CDD9E5"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00D4A017"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="26">
     <fill>
@@ -528,7 +533,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -761,6 +766,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4091,9 +4099,9 @@
       <c r="Q25" s="40" t="inlineStr"/>
       <c r="R25" s="40" t="inlineStr"/>
       <c r="S25" s="40" t="inlineStr"/>
-      <c r="T25" s="38" t="inlineStr">
-        <is>
-          <t>⬜ Pendente</t>
+      <c r="T25" s="42" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
         </is>
       </c>
       <c r="U25" s="41" t="inlineStr">
@@ -4143,9 +4151,9 @@
       <c r="Q26" s="40" t="inlineStr"/>
       <c r="R26" s="40" t="inlineStr"/>
       <c r="S26" s="40" t="inlineStr"/>
-      <c r="T26" s="38" t="inlineStr">
-        <is>
-          <t>⬜ Pendente</t>
+      <c r="T26" s="42" t="inlineStr">
+        <is>
+          <t>✅ Concluido</t>
         </is>
       </c>
       <c r="U26" s="41" t="inlineStr">
@@ -4195,9 +4203,9 @@
       <c r="Q27" s="40" t="inlineStr"/>
       <c r="R27" s="40" t="inlineStr"/>
       <c r="S27" s="40" t="inlineStr"/>
-      <c r="T27" s="38" t="inlineStr">
-        <is>
-          <t>⬜ Pendente</t>
+      <c r="T27" s="42" t="inlineStr">
+        <is>
+          <t>✅ Concluido</t>
         </is>
       </c>
       <c r="U27" s="41" t="inlineStr">
@@ -4247,9 +4255,9 @@
       <c r="Q28" s="40" t="inlineStr"/>
       <c r="R28" s="40" t="inlineStr"/>
       <c r="S28" s="40" t="inlineStr"/>
-      <c r="T28" s="38" t="inlineStr">
-        <is>
-          <t>⬜ Pendente</t>
+      <c r="T28" s="42" t="inlineStr">
+        <is>
+          <t>✅ Concluido</t>
         </is>
       </c>
       <c r="U28" s="41" t="inlineStr"/>
@@ -4295,9 +4303,9 @@
       <c r="Q29" s="40" t="inlineStr"/>
       <c r="R29" s="40" t="inlineStr"/>
       <c r="S29" s="40" t="inlineStr"/>
-      <c r="T29" s="38" t="inlineStr">
-        <is>
-          <t>⬜ Pendente</t>
+      <c r="T29" s="42" t="inlineStr">
+        <is>
+          <t>✅ Concluido</t>
         </is>
       </c>
       <c r="U29" s="41" t="inlineStr">

</xml_diff>

<commit_message>
implementação do back e do end separados
</commit_message>
<xml_diff>
--- a/concursoai_roadmap_v3_FINAL.xlsx
+++ b/concursoai_roadmap_v3_FINAL.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="58">
+  <fonts count="59">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -351,6 +351,11 @@
       <color rgb="008ab0c8"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00FFA500"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="28">
     <fill>
@@ -560,7 +565,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -805,6 +810,7 @@
     <xf numFmtId="0" fontId="55" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5042,9 +5048,9 @@
           <t>💻 Backend</t>
         </is>
       </c>
-      <c r="T48" s="84" t="inlineStr">
-        <is>
-          <t>⬜ Pendente</t>
+      <c r="T48" s="90" t="inlineStr">
+        <is>
+          <t>🟡 Em andamento</t>
         </is>
       </c>
     </row>

</xml_diff>